<commit_message>
feat: implement Teacher module with CRUD operations, DTOs, and enum for teacher type
</commit_message>
<xml_diff>
--- a/recibos/Invoice_Dice_Boy_2025-03-07_19-36.xlsx
+++ b/recibos/Invoice_Dice_Boy_2025-03-07_19-36.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2563C8D4-F2EB-4FE6-A120-D541756AF223}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{567EC904-3251-4461-849D-C14DAF85C53B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8496" yWindow="3132" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Invoice" sheetId="24" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="52">
   <si>
     <t>First Up Consultants</t>
   </si>
@@ -111,6 +111,12 @@
   </si>
   <si>
     <t>Service fee</t>
+  </si>
+  <si>
+    <t>Labor: 5 hours at $75/hr</t>
+  </si>
+  <si>
+    <t>New client discount</t>
   </si>
   <si>
     <t>← The QTY is assumed to be 1 if it is left blank</t>
@@ -1552,20 +1558,20 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:I44"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="7" width="3.75"/>
-    <col min="2" max="2" customWidth="true" style="7" width="40.75"/>
-    <col min="3" max="3" customWidth="true" style="7" width="10.75"/>
-    <col min="4" max="4" customWidth="true" style="7" width="5.75"/>
-    <col min="5" max="6" customWidth="true" style="7" width="18.75"/>
-    <col min="7" max="7" customWidth="true" style="7" width="3.75"/>
+    <col min="1" max="1" customWidth="true" style="7" width="3.796875"/>
+    <col min="2" max="2" customWidth="true" style="7" width="40.796875"/>
+    <col min="3" max="3" customWidth="true" style="7" width="10.796875"/>
+    <col min="4" max="4" customWidth="true" style="7" width="5.796875"/>
+    <col min="5" max="6" customWidth="true" style="7" width="18.796875"/>
+    <col min="7" max="7" customWidth="true" style="7" width="3.796875"/>
     <col min="8" max="8" customWidth="true" style="7" width="29.0"/>
     <col min="9" max="16384" style="7" width="9.0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:9" ht="46.5" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="1" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:9" ht="46.5" customHeight="1" x14ac:dyDescent="0.9">
       <c r="B2" s="52" t="s">
         <v>0</v>
       </c>
@@ -1575,7 +1581,7 @@
       </c>
       <c r="F2" s="60"/>
     </row>
-    <row r="3" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="14" t="s">
         <v>2</v>
       </c>
@@ -1588,7 +1594,7 @@
       </c>
       <c r="I3" s="17"/>
     </row>
-    <row r="4" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="14" t="s">
         <v>4</v>
       </c>
@@ -1601,7 +1607,7 @@
       </c>
       <c r="I4" s="19"/>
     </row>
-    <row r="5" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="14" t="s">
         <v>6</v>
       </c>
@@ -1609,13 +1615,13 @@
       <c r="D5" s="21"/>
       <c r="H5" s="22"/>
     </row>
-    <row r="6" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="23"/>
       <c r="C6" s="18"/>
       <c r="D6" s="24"/>
       <c r="H6" s="22"/>
     </row>
-    <row r="7" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="62" t="s">
         <v>9</v>
       </c>
@@ -1631,9 +1637,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="25" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C8" s="20"/>
       <c r="D8" s="26"/>
@@ -1642,13 +1648,13 @@
       </c>
       <c r="F8" s="27">
         <f ca="1">TODAY()</f>
-        <v>45882</v>
+        <v>45880</v>
       </c>
       <c r="H8" s="22"/>
     </row>
-    <row r="9" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="25" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C9" s="20"/>
       <c r="D9" s="18"/>
@@ -1656,9 +1662,9 @@
       <c r="F9" s="27"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="25" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C10" s="20"/>
       <c r="D10" s="18"/>
@@ -1670,9 +1676,9 @@
       </c>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="25" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C11" s="20"/>
       <c r="D11" s="18"/>
@@ -1686,9 +1692,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="25" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C12" s="20"/>
       <c r="D12" s="18"/>
@@ -1698,9 +1704,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C13" s="18"/>
       <c r="D13" s="18"/>
@@ -1710,7 +1716,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="25"/>
       <c r="C14" s="20"/>
       <c r="D14" s="18"/>
@@ -1720,7 +1726,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="2:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="53" t="s">
         <v>24</v>
       </c>
@@ -1736,9 +1742,9 @@
       </c>
       <c r="H15" s="30"/>
     </row>
-    <row r="16" spans="2:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="31" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C16" s="32"/>
       <c r="D16" s="33" t="n">
@@ -1753,36 +1759,52 @@
       </c>
       <c r="H16" s="22"/>
     </row>
-    <row r="17" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="36"/>
+    <row r="17" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="36" t="s">
+        <v>29</v>
+      </c>
       <c r="C17" s="37"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="40"/>
+      <c r="D17" s="38">
+        <v>5</v>
+      </c>
+      <c r="E17" s="39">
+        <v>75</v>
+      </c>
+      <c r="F17" s="40">
+        <f t="shared" ref="F17:F30" si="0">IF(D17="",ROUND(1*E17,2),ROUND(D17*E17,2))</f>
+        <v>375</v>
+      </c>
       <c r="H17" s="22"/>
     </row>
-    <row r="18" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="36"/>
+    <row r="18" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="36" t="s">
+        <v>30</v>
+      </c>
       <c r="C18" s="37"/>
       <c r="D18" s="38"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="40"/>
+      <c r="E18" s="39">
+        <v>-50</v>
+      </c>
+      <c r="F18" s="40">
+        <f t="shared" si="0"/>
+        <v>-50</v>
+      </c>
       <c r="H18" s="22" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="36"/>
       <c r="C19" s="37"/>
       <c r="D19" s="38"/>
       <c r="E19" s="39"/>
       <c r="F19" s="40">
-        <f t="shared" ref="F17:F30" si="0">IF(D19="",ROUND(1*E19,2),ROUND(D19*E19,2))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H19" s="30"/>
     </row>
-    <row r="20" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="36"/>
       <c r="C20" s="37"/>
       <c r="D20" s="38"/>
@@ -1793,7 +1815,7 @@
       </c>
       <c r="H20" s="30"/>
     </row>
-    <row r="21" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="36"/>
       <c r="C21" s="37"/>
       <c r="D21" s="38"/>
@@ -1804,7 +1826,7 @@
       </c>
       <c r="H21" s="30"/>
     </row>
-    <row r="22" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="36"/>
       <c r="C22" s="37"/>
       <c r="D22" s="38"/>
@@ -1815,7 +1837,7 @@
       </c>
       <c r="H22" s="30"/>
     </row>
-    <row r="23" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="36"/>
       <c r="C23" s="37"/>
       <c r="D23" s="38"/>
@@ -1826,7 +1848,7 @@
       </c>
       <c r="H23" s="30"/>
     </row>
-    <row r="24" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="36"/>
       <c r="C24" s="37"/>
       <c r="D24" s="38"/>
@@ -1837,7 +1859,7 @@
       </c>
       <c r="H24" s="30"/>
     </row>
-    <row r="25" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="36"/>
       <c r="C25" s="37"/>
       <c r="D25" s="38"/>
@@ -1848,7 +1870,7 @@
       </c>
       <c r="H25" s="30"/>
     </row>
-    <row r="26" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="36"/>
       <c r="C26" s="37"/>
       <c r="D26" s="38"/>
@@ -1859,7 +1881,7 @@
       </c>
       <c r="H26" s="30"/>
     </row>
-    <row r="27" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="36"/>
       <c r="C27" s="37"/>
       <c r="D27" s="38"/>
@@ -1870,7 +1892,7 @@
       </c>
       <c r="H27" s="30"/>
     </row>
-    <row r="28" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="36"/>
       <c r="C28" s="37"/>
       <c r="D28" s="38"/>
@@ -1881,7 +1903,7 @@
       </c>
       <c r="H28" s="30"/>
     </row>
-    <row r="29" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="36"/>
       <c r="C29" s="37"/>
       <c r="D29" s="38"/>
@@ -1892,7 +1914,7 @@
       </c>
       <c r="H29" s="30"/>
     </row>
-    <row r="30" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="41"/>
       <c r="C30" s="42"/>
       <c r="D30" s="38"/>
@@ -1903,53 +1925,53 @@
       </c>
       <c r="H30" s="30"/>
     </row>
-    <row r="31" spans="2:8" s="8" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:8" s="8" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="63" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C31" s="63"/>
       <c r="D31" s="64" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E31" s="64"/>
       <c r="F31" s="45">
         <f>SUM(F16:F30)</f>
-        <v>200</v>
+        <v>525</v>
       </c>
       <c r="H31" s="22"/>
     </row>
-    <row r="32" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="23"/>
       <c r="C32" s="16"/>
       <c r="D32" s="64" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E32" s="64"/>
       <c r="F32" s="46">
         <v>4.2500000000000003E-2</v>
       </c>
       <c r="H32" s="22" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="33" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="23"/>
       <c r="C33" s="16"/>
       <c r="D33" s="23" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E33" s="23"/>
       <c r="F33" s="45">
         <f>F31*F32</f>
-        <v>8.5</v>
+        <v>22.3125</v>
       </c>
       <c r="H33" s="22"/>
     </row>
-    <row r="34" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="47"/>
       <c r="C34" s="48"/>
       <c r="D34" s="49" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E34" s="57"/>
       <c r="F34" s="58" t="n">
@@ -1957,20 +1979,20 @@
         <v>2000.0</v>
       </c>
       <c r="H34" s="22" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="35" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="18"/>
       <c r="C35" s="16"/>
       <c r="D35" s="50"/>
       <c r="E35" s="50"/>
       <c r="F35" s="50"/>
       <c r="H35" s="22" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="36" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="36" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="16"/>
       <c r="C36" s="16"/>
       <c r="D36" s="16"/>
@@ -1978,9 +2000,9 @@
       <c r="F36" s="16"/>
       <c r="H36" s="22"/>
     </row>
-    <row r="37" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="65" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C37" s="65"/>
       <c r="D37" s="65"/>
@@ -1988,26 +2010,26 @@
       <c r="F37" s="65"/>
       <c r="H37" s="30"/>
     </row>
-    <row r="38" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="61" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C38" s="61"/>
       <c r="D38" s="61"/>
       <c r="E38" s="61"/>
       <c r="F38" s="61"/>
       <c r="H38" s="22" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="39" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="39" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H39" s="51"/>
     </row>
-    <row r="40" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="2:8" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="41" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="42" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="43" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="44" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="E2:F2"/>
@@ -2041,42 +2063,42 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="1" width="78.75"/>
+    <col min="1" max="1" customWidth="true" style="1" width="78.69921875"/>
     <col min="2" max="16384" style="2" width="9.0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="46.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:2" s="6" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="46.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:2" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">
       <c r="A2" s="59" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="11"/>
     </row>
-    <row r="3" spans="1:2" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="10"/>
     </row>
-    <row r="4" spans="1:2" ht="25.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:2" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:2" ht="25.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:2" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="9"/>
     </row>
-    <row r="8" spans="1:2" ht="82.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -2091,6 +2113,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="30" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cec0622158e8f13124e9e8fd4de31bd1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3b52f30ab005d15df08657af532e6e38" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -2408,15 +2439,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2438,6 +2460,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C42C6076-3E7F-4885-A017-B36671B5853A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{368254F9-4B70-4B70-9250-7541232C303C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2458,14 +2488,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C42C6076-3E7F-4885-A017-B36671B5853A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D626D1C8-EC9A-4213-BF72-F97E82B4EAAA}">
   <ds:schemaRefs>

</xml_diff>